<commit_message>
mejoras de sguridad, rendimiento, ruidio visual
</commit_message>
<xml_diff>
--- a/Cotizador.xlsx
+++ b/Cotizador.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minec\Documents\Catalogos Restaurantes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minec\Documents\Catalogos-Restaurantes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CCF51DA-EA5A-4DC2-A341-BA5660A1F429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF404CB-6E98-4A6F-BE83-F28EA5F8893C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Cotizador_OchentaVeinte_ROI" sheetId="1" r:id="rId1"/>
+    <sheet name="Cotizador_Catalogos" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -125,7 +125,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -188,7 +188,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -237,7 +237,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="166" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="164" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>
@@ -256,7 +256,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="166" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
+      <numFmt numFmtId="164" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>

</xml_diff>

<commit_message>
precios de lanzamiento 2026: Estandar Q299->Q199, Premium Q599->Q349
Sin clientes aun, se baja toda la escalera para quedar dentro de la
banda real del mercado guatemalteco (Q200-Q475). Pro se reubica a
Q599 (sigue pausado). Migracion 111 reconcilia platform_settings;
falta correrla en produccion via SQL Editor de Supabase.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cotizador.xlsx
+++ b/Cotizador.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>599</v>
+        <v>349</v>
       </c>
       <c r="C19" s="4">
         <f>B19*12</f>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>299</v>
+        <v>199</v>
       </c>
       <c r="C19" s="4">
         <f>B19*12</f>

</xml_diff>